<commit_message>
Added excel 1 and excel 2
</commit_message>
<xml_diff>
--- a/S26/MIS_301H/assignments/excel-1/Assignment1_Dawson_Zhang.xlsx
+++ b/S26/MIS_301H/assignments/excel-1/Assignment1_Dawson_Zhang.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dawson/Documents/Classes/S26/MIS_301H/assignments/excel-1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51D117BE-BFFE-E740-A50D-0805A86D5D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACB237BE-5308-784E-B5BA-AC1BE392168E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="26240" windowHeight="15680" activeTab="2" xr2:uid="{2C2D0844-7ACD-4435-B1A8-5F5F49E41FDB}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="3" xr2:uid="{2C2D0844-7ACD-4435-B1A8-5F5F49E41FDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Main Analysis" sheetId="10" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId5"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -430,9 +430,9 @@
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="172" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -455,12 +455,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -633,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -674,25 +668,24 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
@@ -988,40 +981,40 @@
                 <c:formatCode>_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>1863601</c:v>
+                  <c:v>1889994</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>275030</c:v>
+                  <c:v>304325</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>156513</c:v>
+                  <c:v>165966.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>127750</c:v>
+                  <c:v>131372</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>189012</c:v>
+                  <c:v>170478</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>335119.8</c:v>
+                  <c:v>301000</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>204960</c:v>
+                  <c:v>211496</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>37662.5</c:v>
+                  <c:v>37125</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>404745</c:v>
+                  <c:v>417840</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>200472</c:v>
+                  <c:v>209371.08</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>226880</c:v>
+                  <c:v>226200</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>260300</c:v>
+                  <c:v>268825</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1072,40 +1065,40 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>12.938676140613314</c:v>
+                  <c:v>13.136080777860883</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.7053892215568864</c:v>
+                  <c:v>4.206586826347305</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.9714031971580819</c:v>
+                  <c:v>3.2112788632326819</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.9615634272997033</c:v>
+                  <c:v>2.0455304154302669</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.1063118480877241</c:v>
+                  <c:v>0.89977266648836585</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.3614236902050108</c:v>
+                  <c:v>4.7137433561123769</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.94046807543740063</c:v>
+                  <c:v>1.0023479512232067</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-0.46387900355871886</c:v>
+                  <c:v>-0.47153024911032027</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.7239047042196649</c:v>
+                  <c:v>1.8120331112457098</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.75152023485007335</c:v>
+                  <c:v>0.82927133570979228</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.4779379641764963</c:v>
+                  <c:v>1.4705111402359108</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.1189773844641104</c:v>
+                  <c:v>4.2866273352999018</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1175,6 +1168,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1592384960"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -1233,6 +1227,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1592384064"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
@@ -1288,6 +1283,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1604565440"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -1498,19 +1494,19 @@
                 <c:formatCode>_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* "-"??_);_(@_)</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1795962.7600000002</c:v>
+                  <c:v>1802146.96</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1934150.88</c:v>
+                  <c:v>1935756.6400000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1584988.87</c:v>
+                  <c:v>1582359.1300000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1486223.6799999997</c:v>
+                  <c:v>1465187.4879999999</c:v>
                 </c:pt>
                 <c:pt idx="4" formatCode="&quot;$&quot;#,##0.00">
-                  <c:v>4283603.3</c:v>
+                  <c:v>4335550.58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1561,19 +1557,19 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.79613124525543355</c:v>
+                  <c:v>0.80214695999999996</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.93433610278901702</c:v>
+                  <c:v>0.93575664000000014</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.58507874394585768</c:v>
+                  <c:v>0.58235913000000017</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.48622422457113135</c:v>
+                  <c:v>0.46518748799999987</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.2836032999999998</c:v>
+                  <c:v>3.33555058</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1643,6 +1639,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1752142656"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -1701,6 +1698,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1622648448"/>
+        <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:valAx>
@@ -1756,6 +1754,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="1566880000"/>
+        <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
@@ -3107,13 +3106,13 @@
     <cacheField name="Total Purchase Value " numFmtId="44">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="39410" maxValue="148590"/>
     </cacheField>
-    <cacheField name="Current Price" numFmtId="172">
+    <cacheField name="Current Price" numFmtId="165">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="15.035" maxValue="473.82"/>
     </cacheField>
-    <cacheField name="Total Current Value" numFmtId="172">
+    <cacheField name="Total Current Value" numFmtId="165">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="37587.5" maxValue="1867649.9999999998"/>
     </cacheField>
-    <cacheField name="Gain  (Loss) " numFmtId="172">
+    <cacheField name="Gain  (Loss) " numFmtId="165">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="-32662.5" maxValue="1733949.9999999998"/>
     </cacheField>
     <cacheField name="Percent Gain (Loss)  " numFmtId="10">
@@ -3298,7 +3297,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{ABD18DCA-C566-0644-8D09-5710E139509E}" name="PivotTable2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{ABD18DCA-C566-0644-8D09-5710E139509E}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:D6" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -3314,9 +3313,9 @@
     <pivotField numFmtId="44" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" numFmtId="44" showAll="0"/>
-    <pivotField numFmtId="172" showAll="0"/>
-    <pivotField dataField="1" numFmtId="172" showAll="0"/>
-    <pivotField dataField="1" numFmtId="172" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField dataField="1" numFmtId="165" showAll="0"/>
+    <pivotField dataField="1" numFmtId="165" showAll="0"/>
     <pivotField numFmtId="10" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -3349,8 +3348,8 @@
   </colItems>
   <dataFields count="3">
     <dataField name="Sum of Total Purchase Value " fld="6" baseField="0" baseItem="0" numFmtId="44"/>
-    <dataField name="Sum of Total Current Value" fld="8" baseField="0" baseItem="0" numFmtId="172"/>
-    <dataField name="Sum of Gain  (Loss) " fld="9" baseField="0" baseItem="0" numFmtId="172"/>
+    <dataField name="Sum of Total Current Value" fld="8" baseField="0" baseItem="0" numFmtId="165"/>
+    <dataField name="Sum of Gain  (Loss) " fld="9" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -3370,7 +3369,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79D67C0A-51C4-764A-ADD3-A98CB0DA0337}" name="PivotTable1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79D67C0A-51C4-764A-ADD3-A98CB0DA0337}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:D10" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0">
@@ -3428,9 +3427,9 @@
     <pivotField numFmtId="44" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField dataField="1" numFmtId="44" showAll="0"/>
-    <pivotField numFmtId="172" showAll="0"/>
-    <pivotField dataField="1" numFmtId="172" showAll="0"/>
-    <pivotField dataField="1" numFmtId="172" showAll="0"/>
+    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField dataField="1" numFmtId="165" showAll="0"/>
+    <pivotField dataField="1" numFmtId="165" showAll="0"/>
     <pivotField numFmtId="10" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -3475,8 +3474,8 @@
   </colItems>
   <dataFields count="3">
     <dataField name="Sum of Total Purchase Value " fld="6" baseField="0" baseItem="0" numFmtId="44"/>
-    <dataField name="Sum of Total Current Value" fld="8" baseField="0" baseItem="0" numFmtId="172"/>
-    <dataField name="Sum of Gain  (Loss) " fld="9" baseField="0" baseItem="0" numFmtId="172"/>
+    <dataField name="Sum of Total Current Value" fld="8" baseField="0" baseItem="0" numFmtId="165"/>
+    <dataField name="Sum of Gain  (Loss) " fld="9" baseField="0" baseItem="0" numFmtId="165"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -3644,9 +3643,9 @@
     <v>Powered by Refinitiv</v>
     <v>212.18989999999999</v>
     <v>86.62</v>
-    <v>2.3111000000000002</v>
-    <v>-1.3099000000000001</v>
-    <v>-6.9799999999999992E-3</v>
+    <v>2.3109000000000002</v>
+    <v>-2.1305999999999998</v>
+    <v>-1.1147000000000001E-2</v>
     <v>USD</v>
     <v>NVIDIA Corporation is a full-stack computing infrastructure company. The Company is engaged in accelerated computing to help solve the challenging computational problems. The Company’s segments include Compute &amp; Networking and Graphics. The Compute &amp; Networking segment includes its Data Center accelerated computing platforms and artificial intelligence (AI) solutions and software; networking; automotive platforms and autonomous and electric vehicle solutions; Jetson for robotics and other embedded platforms, and DGX Cloud computing services. The Graphics segment includes GeForce GPUs for gaming and PCs, the GeForce NOW game streaming service and related infrastructure, and solutions for gaming platforms; Quadro/NVIDIA RTX GPUs for enterprise workstation graphics; virtual GPU software for cloud-based visual and virtual computing; automotive platforms for infotainment systems, and Omniverse Enterprise software for building and operating industrial AI and digital twin applications.</v>
     <v>36000</v>
@@ -3654,24 +3653,24 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>2788 San Tomas Expressway, SANTA CLARA, CA, 95051 US</v>
-    <v>189.12</v>
+    <v>189.38</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>Stock</v>
-    <v>46048.833629825778</v>
+    <v>46055.684842742972</v>
     <v>0</v>
-    <v>185.99</v>
-    <v>4528550430000</v>
+    <v>186.42</v>
+    <v>4592685420000</v>
     <v>NVIDIA CORPORATION</v>
     <v>NVIDIA CORPORATION</v>
-    <v>187.14</v>
-    <v>46.157299999999999</v>
-    <v>187.67</v>
-    <v>186.36009999999999</v>
+    <v>187.23</v>
+    <v>46.811</v>
+    <v>191.13</v>
+    <v>188.99940000000001</v>
     <v>24300000000</v>
     <v>NVDA</v>
     <v>NVIDIA CORPORATION (XNAS:NVDA)</v>
-    <v>90270606</v>
-    <v>163788356</v>
+    <v>56019045</v>
+    <v>153411649</v>
     <v>1998</v>
   </rv>
   <rv s="2">
@@ -3693,36 +3692,36 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>412.42989999999998</v>
+    <v>455.5</v>
     <v>61.54</v>
-    <v>1.5081</v>
-    <v>-6.75</v>
-    <v>-1.6890000000000002E-2</v>
+    <v>1.5076000000000001</v>
+    <v>19.87</v>
+    <v>4.7892999999999998E-2</v>
     <v>USD</v>
-    <v>Micron Technology, Inc. provides memory and storage solutions. The Company delivers a portfolio of high-performance dynamic random-access memory (DRAM), NAND, and NOR memory and storage products through its Micron and Crucial brands. The Company's products enable advancing in artificial intelligence (AI) and compute-intensive applications. Its segments include Cloud Memory Business Unit (CMBU), Core Data Center Business Unit (CDBU), Mobile and Client Business Unit (MCBU) and Automotive and Embedded Business Unit (AEBU). CMBU is focused on memory solutions for large hyperscale cloud customers, and high bandwidth memory (HBM) for all data center customers. CDBU is focused on memory solutions for mid-tier cloud, enterprise, and OEM data center customers and storage solutions for all data center customers. MCBU is focused on memory and storage solutions for mobile and client segments. AEBU is focused on memory and storage solutions for the automotive, industrial, and consumer segments.</v>
+    <v>Micron Technology, Inc. provides memory and storage solutions. The Company delivers a portfolio of high-performance dynamic random-access memory (DRAM), NAND, and NOR memory and storage products through its Micron and Crucial brands. The Company's products enable advancing in artificial intelligence (AI) and compute-intensive applications. Its segments include Compute and Networking Business Unit (CNBU), Mobile Business Unit (MBU), Embedded Business Unit (EBU), and Storage Business Unit (SBU). CNBU segment includes memory products and solutions sold into the data center, PC, graphics, and networking markets. MBU segment includes memory and storage products sold into the smartphone and other mobile-device markets. EBU segment includes memory and storage products and solutions sold into the intelligent edge through the automotive, industrial, and consumer embedded markets. SBU segment includes SSDs and component-level storage solutions sold into the data center, PC, and consumer markets.</v>
     <v>53000</v>
     <v>Nasdaq Stock Market</v>
     <v>XNAS</v>
     <v>XNAS</v>
     <v>8000 S Federal Way, Po Box 6, BOISE, ID, 83716-9632 US</v>
-    <v>398</v>
+    <v>436.7</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>Stock</v>
-    <v>46048.833622164064</v>
+    <v>46055.684840890623</v>
     <v>3</v>
-    <v>384.3</v>
-    <v>442212486100</v>
+    <v>410</v>
+    <v>489315037750</v>
     <v>MICRON TECHNOLOGY, INC.</v>
     <v>MICRON TECHNOLOGY, INC.</v>
-    <v>395.41</v>
-    <v>37.347900000000003</v>
-    <v>399.65</v>
-    <v>392.9</v>
+    <v>412.13</v>
+    <v>41.326000000000001</v>
+    <v>414.88</v>
+    <v>434.75</v>
     <v>1125509000</v>
     <v>MU</v>
     <v>MICRON TECHNOLOGY, INC. (XNAS:MU)</v>
-    <v>23238822</v>
-    <v>34912533</v>
+    <v>18502788</v>
+    <v>34145551</v>
     <v>1984</v>
   </rv>
   <rv s="2">
@@ -3744,11 +3743,11 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>236.1</v>
+    <v>251.87</v>
     <v>56.32</v>
-    <v>1.7827</v>
-    <v>5.65</v>
-    <v>2.5924999999999997E-2</v>
+    <v>1.7818000000000001</v>
+    <v>3.6349999999999998</v>
+    <v>1.5569999999999999E-2</v>
     <v>USD</v>
     <v>Lam Research Corporation is a global supplier of wafer fabrication equipment and services to the semiconductor industry. The Company designs, manufactures, markets, refurbishes, and services semiconductor processing equipment used in the fabrication of integrated circuits. Its products and services are designed to help its customers build devices that are used in a variety of electronic products, including mobile phones, personal computers, servers, wearables, automotive vehicles, and data storage devices. Its product families include ALTUS, SABRE, SPEED, Striker, VECTOR, Flex, Vantex, Kiyo, Versys Metal, Syndion, Coronus, and DV-Prime, Da Vinci, EOS, and SP Series. Its customer base includes semiconductor memory, foundries, and integrated device manufacturers that make products such as non-volatile memory, dynamic random-access memory, and logic devices. It offers services in areas, such as nanoscale applications enablement, chemistry, plasma and fluidics, and others.</v>
     <v>19000</v>
@@ -3756,24 +3755,24 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>4650 Cushing Blvd, FREMONT, CA, 94538 US</v>
-    <v>225.35</v>
+    <v>242.95</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>Stock</v>
-    <v>46048.833619930469</v>
+    <v>46055.684821180468</v>
     <v>6</v>
-    <v>215.93010000000001</v>
-    <v>280835747700</v>
+    <v>232</v>
+    <v>296077360245</v>
     <v>LAM RESEARCH CORPORATION</v>
     <v>LAM RESEARCH CORPORATION</v>
-    <v>218.98</v>
-    <v>49.2684</v>
-    <v>217.94</v>
-    <v>223.59</v>
-    <v>1256030000</v>
+    <v>233</v>
+    <v>48.591999999999999</v>
+    <v>233.46</v>
+    <v>237.095</v>
+    <v>1248771000</v>
     <v>LRCX</v>
     <v>LAM RESEARCH CORPORATION (XNAS:LRCX)</v>
-    <v>6402017</v>
-    <v>12723578</v>
+    <v>4972756</v>
+    <v>12353333</v>
     <v>1989</v>
   </rv>
   <rv s="2">
@@ -3795,11 +3794,11 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>333.03</v>
+    <v>344.6</v>
     <v>123.73650000000001</v>
     <v>1.6941999999999999</v>
-    <v>-3.0049999999999999</v>
-    <v>-9.3210000000000012E-3</v>
+    <v>6.11</v>
+    <v>1.8956000000000001E-2</v>
     <v>USD</v>
     <v>Applied Materials, Inc. is a materials engineering solution company. The Company provides equipment, services and software to the semiconductor, display, and related industries. It operates in three segments: Semiconductor Systems, Applied Global Services (AGS), and Display. The Semiconductor systems segment designs, develops, manufactures and sells a range of primarily 300 mm equipment used to fabricate semiconductor chips, also referred to as integrated circuits (ICs). The AGS segment provides services, spares and factory automation software to customer fabrication plants globally. The AGS segment also manufactures and sells 200mm and other equipment. The Display segment is comprised primarily of products for manufacturing liquid crystal displays (LCDs), organic light-emitting diodes (OLEDs), and other display technologies for televisions, monitors, laptops, personal computers (PCs), tablets, smartphones, and other consumer-oriented devices.</v>
     <v>36500</v>
@@ -3807,24 +3806,24 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>3050 Bowers Avenue, P.O. Box 58039, SANTA CLARA, CA, 95054-3299 US</v>
-    <v>322</v>
+    <v>330.44</v>
     <v>Semiconductors &amp; Semiconductor Equipment</v>
     <v>Stock</v>
-    <v>46048.833623251565</v>
+    <v>46055.684808935155</v>
     <v>9</v>
-    <v>316.57</v>
-    <v>253246298375</v>
+    <v>319.85000000000002</v>
+    <v>260681919402</v>
     <v>APPLIED MATERIALS, INC.</v>
     <v>APPLIED MATERIALS, INC.</v>
-    <v>322</v>
-    <v>36.832099999999997</v>
-    <v>322.38</v>
-    <v>319.375</v>
-    <v>792943400</v>
+    <v>322.11</v>
+    <v>37.876399999999997</v>
+    <v>322.32</v>
+    <v>328.43</v>
+    <v>793721400</v>
     <v>AMAT</v>
     <v>APPLIED MATERIALS, INC. (XNAS:AMAT)</v>
-    <v>2744217</v>
-    <v>7200774</v>
+    <v>2556181</v>
+    <v>6725771</v>
     <v>1987</v>
   </rv>
   <rv s="2">
@@ -3868,9 +3867,9 @@
     <v>Powered by Refinitiv</v>
     <v>555.45000000000005</v>
     <v>344.79</v>
-    <v>1.0841000000000001</v>
-    <v>6.58</v>
-    <v>1.4121999999999999E-2</v>
+    <v>1.0848</v>
+    <v>-4.0949999999999998</v>
+    <v>-9.5169999999999994E-3</v>
     <v>USD</v>
     <v>Microsoft Corporation is a technology company that develops and supports software, services, devices, and solutions. Its Productivity and Business Processes segment consists of products and services in its portfolio of productivity, communication, and information services, spanning a variety of devices and platforms. It comprises Microsoft 365 Commercial products and cloud services; Microsoft 365 Consumer products and cloud services; LinkedIn, and Dynamics products and cloud services. The Intelligent Cloud segment consists of its public, private, and hybrid server products and cloud services. It comprises server products and cloud services, including Azure, and enterprise and partner services, including Enterprise Support Services. Its More Personal Computing segment primarily comprises Windows and Devices, including Windows OEM licensing; Gaming, including Xbox hardware and Xbox content; Search and news advertising, comprising Bing and Copilot, Microsoft News, and Microsoft Edge.</v>
     <v>228000</v>
@@ -3878,25 +3877,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Microsoft Way, REDMOND, WA, 98052 US</v>
-    <v>474.25</v>
+    <v>430.73599999999999</v>
     <v>15</v>
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
-    <v>46048.833641978905</v>
+    <v>46055.684855428124</v>
     <v>16</v>
-    <v>462</v>
-    <v>3512021103810</v>
+    <v>424.52</v>
+    <v>3164765951655</v>
     <v>MICROSOFT CORPORATION</v>
     <v>MICROSOFT CORPORATION</v>
-    <v>465</v>
-    <v>33.619100000000003</v>
-    <v>465.95</v>
-    <v>472.53</v>
-    <v>7432377000</v>
+    <v>430.23</v>
+    <v>26.666499999999999</v>
+    <v>430.29</v>
+    <v>426.19499999999999</v>
+    <v>7425629000</v>
     <v>MSFT</v>
     <v>MICROSOFT CORPORATION (XNAS:MSFT)</v>
-    <v>17166806</v>
-    <v>24479233</v>
+    <v>14030134</v>
+    <v>29568004</v>
     <v>1993</v>
   </rv>
   <rv s="2">
@@ -3920,9 +3919,9 @@
     <v>Powered by Refinitiv</v>
     <v>207.52</v>
     <v>66.12</v>
-    <v>1.6409</v>
-    <v>-2.0400999999999998</v>
-    <v>-1.2029000000000001E-2</v>
+    <v>1.6422000000000001</v>
+    <v>3.91</v>
+    <v>2.6672999999999999E-2</v>
     <v>USD</v>
     <v>Palantir Technologies Inc. is engaged in building software to assist in counterterrorism investigations and operations. The Company has built four principal software platforms, including Palantir Gotham (Gotham), Palantir Foundry (Foundry), Palantir Apollo (Apollo), and Palantir Artificial Intelligence Platform (AIP). Apollo is a cloud-agnostic, single control layer that coordinates ongoing delivery of new features, security updates, and platform configurations, helping to ensure the continuous operation of critical systems. Gotham enables users to identify patterns hidden deep within datasets, ranging from signals intelligence sources to reports from confidential informants. Foundry transforms the ways organizations operate by creating a central operating system for their data. AIP enables responsible artificial intelligence (AI)-advantage across the enterprise by using primary, core components built to effectively activate large language models and other AI within any organization.</v>
     <v>4414</v>
@@ -3930,24 +3929,24 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>1200 17Th Street, Floor 15, DENVER, CO, 80202 US</v>
-    <v>170.58969999999999</v>
+    <v>151.4</v>
     <v>Software &amp; IT Services</v>
     <v>Stock</v>
-    <v>46048.833629872657</v>
+    <v>46055.684840520313</v>
     <v>19</v>
-    <v>167.4068</v>
-    <v>399199900116</v>
+    <v>148.08000000000001</v>
+    <v>358555865500</v>
     <v>PALANTIR TECHNOLOGIES INC.</v>
     <v>PALANTIR TECHNOLOGIES INC.</v>
-    <v>168.21</v>
-    <v>391.86130000000003</v>
-    <v>169.6</v>
-    <v>167.5599</v>
+    <v>151.13999999999999</v>
+    <v>351.96449999999999</v>
+    <v>146.59</v>
+    <v>150.5</v>
     <v>2382431000</v>
     <v>PLTR</v>
     <v>PALANTIR TECHNOLOGIES INC. (XNAS:PLTR)</v>
-    <v>17177058</v>
-    <v>37206555</v>
+    <v>21539777</v>
+    <v>36124862</v>
     <v>2003</v>
   </rv>
   <rv s="2">
@@ -3971,9 +3970,9 @@
     <v>Powered by Refinitiv</v>
     <v>288.62</v>
     <v>169.21010000000001</v>
-    <v>1.0951</v>
-    <v>8.16</v>
-    <v>3.2898000000000004E-2</v>
+    <v>1.0946</v>
+    <v>4.8899999999999997</v>
+    <v>1.8845000000000001E-2</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, and Wearables, Home and Accessories. Its software platforms include iOS, iPadOS, macOS, watchOS, visionOS, and tvOS. Its services include advertising, AppleCare, cloud services, digital content and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -3981,24 +3980,24 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>256.56</v>
+    <v>265.37</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46048.833636978903</v>
+    <v>46055.684834640626</v>
     <v>22</v>
-    <v>249.8</v>
-    <v>3765609666000</v>
+    <v>259.20499999999998</v>
+    <v>3886952799000</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>251.45</v>
-    <v>34.497599999999998</v>
-    <v>248.04</v>
-    <v>256.2</v>
-    <v>14697930000</v>
+    <v>260.02999999999997</v>
+    <v>33.587400000000002</v>
+    <v>259.48</v>
+    <v>264.37</v>
+    <v>14702700000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>33221155</v>
-    <v>46344462</v>
+    <v>23600188</v>
+    <v>46103925</v>
     <v>1977</v>
   </rv>
   <rv s="2">
@@ -4022,9 +4021,9 @@
     <v>Powered by Refinitiv</v>
     <v>19.82</v>
     <v>7.625</v>
-    <v>2.0548999999999999</v>
-    <v>0.155</v>
-    <v>1.0396000000000001E-2</v>
+    <v>2.0552000000000001</v>
+    <v>0.5</v>
+    <v>3.4842999999999999E-2</v>
     <v>USD</v>
     <v>Sonos, Inc., and its wholly owned subsidiaries designs, develops, manufactures, and sells audio products and services. It offers customers a proprietary software platform, and the ability to stream content from a variety of sources over the customer’s wireless network or over Bluetooth. Its product lineup includes wireless, portable, and home theater speakers, headphones, components, and accessories. Its products are sold through third-party physical retailers, including custom installers of home audio systems, e-commerce retailers, and its Website sonos.com. Its products include Era 100, Era 300, Five, Roam 2, Move 2, Ray, Beam (Gen 2), Arc, Sub Mini, and Sub (Gen 3). Its proprietary software includes multi-room, multi-service experience, open platform for content partners, and smart audio tuning. Its products are distributed in more than 60 countries through retailer's physical stores and their websites, online retailers, custom installers who bundle its products with their services.</v>
     <v>1404</v>
@@ -4032,24 +4031,24 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>301 Coromar Drive, SANTA BARBARA, CA, 93117 US</v>
-    <v>15.32</v>
+    <v>15</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46048.833566307811</v>
+    <v>46055.684831874998</v>
     <v>25</v>
-    <v>14.62</v>
-    <v>1820947225</v>
+    <v>14.22</v>
+    <v>1794959595</v>
     <v>SONOS, INC.</v>
     <v>SONOS, INC.</v>
-    <v>14.86</v>
+    <v>14.43</v>
     <v>0</v>
-    <v>14.91</v>
-    <v>15.065</v>
+    <v>14.35</v>
+    <v>14.85</v>
     <v>120872700</v>
     <v>SONO</v>
     <v>SONOS, INC. (XNAS:SONO)</v>
-    <v>818138</v>
-    <v>1370047</v>
+    <v>358290</v>
+    <v>1259070</v>
     <v>2002</v>
   </rv>
   <rv s="2">
@@ -4071,11 +4070,11 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>136.93979999999999</v>
+    <v>142.34</v>
     <v>97.8</v>
-    <v>0.3795</v>
-    <v>-5.5E-2</v>
-    <v>-4.0750000000000004E-4</v>
+    <v>0.379</v>
+    <v>-2.12</v>
+    <v>-1.4993000000000001E-2</v>
     <v>USD</v>
     <v>Exxon Mobil Corporation is an energy provider and chemical manufacturer. The Company’s principal business involves exploration for, and production of, crude oil and natural gas; the manufacture, trade, transport and sale of crude oil, natural gas, petroleum products, petrochemicals and a wide variety of specialty products; and pursuit of lower-emission and other new business opportunities, including carbon capture and storage, hydrogen, lower-emission fuels, Proxxima systems, carbon materials, and lithium. Its Upstream segment explores for and produces crude oil and natural gas. The Energy Products, Chemical Products, and Specialty Products segments manufacture and sell petroleum products and petrochemicals. Energy Products segment includes fuels, aromatics, and catalysts and licensing. Chemical Products segment consists of olefins, polyolefins, and intermediates. Specialty Products segment includes finished lubricants, basestocks and waxes, synthetics, and elastomers and resins.</v>
     <v>61000</v>
@@ -4083,24 +4082,24 @@
     <v>XNYS</v>
     <v>XNYS</v>
     <v>22777 SPRINGWOODS VILLAGE PARKWAY, SPRING, TX, 77389-1425 US</v>
-    <v>136.93979999999999</v>
+    <v>140.32</v>
     <v>Oil &amp; Gas</v>
     <v>Stock</v>
-    <v>46048.833626168751</v>
+    <v>46055.684844640622</v>
     <v>28</v>
-    <v>134.16999999999999</v>
-    <v>568958950890</v>
+    <v>138.12010000000001</v>
+    <v>587366880480</v>
     <v>EXXON MOBIL CORPORATION</v>
     <v>EXXON MOBIL CORPORATION</v>
-    <v>136.88</v>
-    <v>19.6114</v>
-    <v>134.97</v>
-    <v>134.91499999999999</v>
+    <v>140</v>
+    <v>20.804200000000002</v>
+    <v>141.4</v>
+    <v>139.28</v>
     <v>4217166000</v>
     <v>XOM</v>
     <v>EXXON MOBIL CORPORATION (XNYS:XOM)</v>
-    <v>8536773</v>
-    <v>17809156</v>
+    <v>5997875</v>
+    <v>18196032</v>
     <v>1882</v>
   </rv>
   <rv s="2">
@@ -4122,11 +4121,11 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>169.37</v>
+    <v>177.3</v>
     <v>132.04</v>
-    <v>0.68840000000000001</v>
-    <v>0.34</v>
-    <v>2.039E-3</v>
+    <v>0.68769999999999998</v>
+    <v>-2.4241000000000001</v>
+    <v>-1.3703E-2</v>
     <v>USD</v>
     <v>Chevron Corporation is an integrated energy company. The Company produces crude oil and natural gas; manufactures transportation fuels, lubricants, petrochemicals and additives; and develops technologies that enhance its business and industry. The Company’s segments include Upstream and Downstream. Upstream operations consist primarily of exploring for, developing, producing and transporting crude oil and natural gas; liquefaction, transportation and regasification associated with LNG; transporting crude oil by major international oil export pipelines; processing, transporting, storage and marketing of natural gas; carbon capture and storage; and a gas-to-liquids plant. Downstream operations consist primarily of the refining of crude oil into petroleum products; marketing crude oil, refined products, and lubricants; manufacturing and marketing of renewable fuels, and transporting of crude oil and refined products by pipeline, marine vessel, motor equipment and rail car.</v>
     <v>45298</v>
@@ -4134,24 +4133,24 @@
     <v>XNYS</v>
     <v>XNYS</v>
     <v>1400 SMITH STREET, HOUSTON, TX, 77002 US</v>
-    <v>168.37</v>
+    <v>175.1069</v>
     <v>Oil &amp; Gas</v>
     <v>Stock</v>
-    <v>46048.833614385934</v>
+    <v>46055.684826249999</v>
     <v>31</v>
-    <v>166.77</v>
-    <v>336378985320</v>
+    <v>172.65</v>
+    <v>351311063119</v>
     <v>CHEVRON CORPORATION</v>
     <v>CHEVRON CORPORATION</v>
-    <v>168.37</v>
-    <v>23.589700000000001</v>
-    <v>166.72</v>
-    <v>167.06</v>
+    <v>173.49</v>
+    <v>26.244900000000001</v>
+    <v>176.9</v>
+    <v>174.4759</v>
     <v>2013522000</v>
     <v>CVX</v>
     <v>CHEVRON CORPORATION (XNYS:CVX)</v>
-    <v>5347871</v>
-    <v>10759592</v>
+    <v>4086398</v>
+    <v>11452315</v>
     <v>1926</v>
   </rv>
   <rv s="2">
@@ -4173,36 +4172,36 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>56.795000000000002</v>
+    <v>58.5</v>
     <v>33.6</v>
-    <v>0.87780000000000002</v>
-    <v>2.8</v>
-    <v>5.1928999999999996E-2</v>
+    <v>0.87739999999999996</v>
+    <v>0.51</v>
+    <v>9.1009999999999997E-3</v>
     <v>USD</v>
-    <v>Baker Hughes Company is an energy technology company that provides solutions to energy and industrial customers worldwide. The Company's segments include Oilfield Services &amp; Equipment (OFSE) and Industrial &amp; Energy Technology (IET). OFSE segment provides products and services for onshore and offshore oilfield operations across the lifecycle of a well, ranging from exploration, appraisal, and development, to production, rejuvenation, and decommissioning. OFSE segment is organized into four product lines: Well Construction; Completions, Intervention, and Measurements; Production Solutions, and Subsea. IET segment provides technology solutions and services for mechanical-drive, compression and power-generation applications across the energy industry including oil and gas, liquefied natural gas operations, downstream refining, and petrochemical markets, as well as lower carbon solutions to broader energy and industrial sectors. IET segment also provides equipment, software, and services.</v>
+    <v>Baker Hughes Company is an energy technology company with a portfolio of technologies and services that span the energy and industrial value chain. The Company operates in two segments: Oilfield Services &amp; Equipment (OFSE) and Industrial &amp; Energy Technology (IET). OFSE segment provides products and services for onshore and offshore oilfield operations across the lifecycle of a well, ranging from exploration, appraisal, and development, to production, rejuvenation, and decommissioning. OFSE is organized into four product lines: Well Construction; Completions, Intervention, and Measurements; Production Solutions, and Subsea and Surface Pressure Systems. IET segment provides technology solutions and services for mechanical-drive, compression and power-generation applications across the energy industry, including oil and gas, liquefied natural gas (LNG) operations, downstream refining and petrochemical markets, as well as lower carbon solutions to broader energy and industrial sectors.</v>
     <v>57000</v>
     <v>Nasdaq Stock Market</v>
     <v>XNAS</v>
     <v>XNAS</v>
     <v>575 NORTH DAIRY ASHFORD ROAD, SUITE 100, HOUSTON, TX, 77079-1121 US</v>
-    <v>56.795000000000002</v>
+    <v>56.72</v>
     <v>Oil &amp; Gas Related Equipment and Services</v>
     <v>Stock</v>
-    <v>46048.833644687496</v>
+    <v>46055.684814328124</v>
     <v>34</v>
-    <v>54.82</v>
-    <v>55969815608</v>
+    <v>55.27</v>
+    <v>55814850000</v>
     <v>BAKER HUGHES COMPANY</v>
     <v>BAKER HUGHES COMPANY</v>
-    <v>55.65</v>
-    <v>19.549900000000001</v>
-    <v>53.92</v>
-    <v>56.72</v>
-    <v>986773900</v>
+    <v>55.77</v>
+    <v>21.719899999999999</v>
+    <v>56.04</v>
+    <v>56.55</v>
+    <v>987000000</v>
     <v>BKR</v>
     <v>BAKER HUGHES COMPANY (XNAS:BKR)</v>
-    <v>11324036</v>
-    <v>8507632</v>
+    <v>1483703</v>
+    <v>9001258</v>
     <v>2016</v>
   </rv>
   <rv s="2">
@@ -4226,9 +4225,9 @@
     <v>Powered by Refinitiv</v>
     <v>59.8</v>
     <v>14.27</v>
-    <v>1.1451</v>
-    <v>-1.64</v>
-    <v>-3.0539999999999998E-2</v>
+    <v>1.1448</v>
+    <v>-1.425</v>
+    <v>-2.5819999999999999E-2</v>
     <v>USD</v>
     <v>Solaris Energy Infrastructure, Inc. provides mobile and scalable equipment-based solutions for use in distributed power generation as well as the management of raw materials used in the completion of oil and natural gas wells. Its segments include Solaris Power Solutions and Solaris Logistics Solutions. The Solaris Power Solutions segment offers configurable sets of natural gas-powered mobile turbines and ancillary equipment. This segment leases equipment to data center and oilfield customers and is focused on continuing to grow its services with these customers as well as across multiple commercial and industrial end-markets. The Solaris Logistics Solutions segment designs and manufactures specialized equipment that enables the management of raw materials used in the completion of oil and natural gas wells. Its equipment-based logistics services include field technician support, software solutions, and also include last mile and mobilization services.</v>
     <v>364</v>
@@ -4236,24 +4235,24 @@
     <v>XNYS</v>
     <v>XNYS</v>
     <v>9651 KATY FREEWAY, SUITE 300, HOUSTON, TX, 77024 US</v>
-    <v>55.25</v>
+    <v>55.44</v>
     <v>Oil &amp; Gas Related Equipment and Services</v>
     <v>Stock</v>
-    <v>46048.833642661717</v>
+    <v>46055.684674385935</v>
     <v>37</v>
-    <v>51.82</v>
-    <v>3563900573</v>
+    <v>52.56</v>
+    <v>3680620713</v>
     <v>SOLARIS ENERGY INFRASTRUCTURE, INC.</v>
     <v>SOLARIS ENERGY INFRASTRUCTURE, INC.</v>
     <v>53.66</v>
-    <v>56.044800000000002</v>
-    <v>53.7</v>
-    <v>52.06</v>
+    <v>57.880299999999998</v>
+    <v>55.19</v>
+    <v>53.765000000000001</v>
     <v>68457560</v>
     <v>SEI</v>
     <v>SOLARIS ENERGY INFRASTRUCTURE, INC. (XNYS:SEI)</v>
-    <v>1674083</v>
-    <v>2363192</v>
+    <v>578208</v>
+    <v>2332355</v>
     <v>2017</v>
   </rv>
   <rv s="2">
@@ -4275,27 +4274,27 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>0.27</v>
-    <v>4.2279999999999998E-4</v>
+    <v>-2.73</v>
+    <v>-4.241E-3</v>
     <v>US</v>
     <v>USD</v>
     <v>1.4000000000000002E-3</v>
     <v>Mutual Fund</v>
-    <v>46045.989583333336</v>
-    <v>46047.461287439066</v>
+    <v>46052.989583333336</v>
+    <v>46053.840996073435</v>
     <v>40</v>
     <v>Vanguard 500 Index Fund;Investor</v>
     <v>2854928268</v>
-    <v>638.55999999999995</v>
-    <v>638.83000000000004</v>
-    <v>4.2236000000000002</v>
-    <v>1.6619999999999998E-3</v>
-    <v>-4.3809999999999995E-3</v>
-    <v>0.14882999999999999</v>
-    <v>3.4733E-2</v>
-    <v>0.213556</v>
-    <v>0.139652</v>
-    <v>1.0903000000000001E-2</v>
+    <v>643.76</v>
+    <v>641.03</v>
+    <v>4.1615000000000002</v>
+    <v>6.9899999999999997E-3</v>
+    <v>3.444E-3</v>
+    <v>0.15604999999999999</v>
+    <v>1.9974000000000002E-2</v>
+    <v>0.21507699999999999</v>
+    <v>0.148089</v>
+    <v>1.4383999999999999E-2</v>
     <v>VFINX</v>
     <v>Vanguard 500 Index Fund;Investor</v>
   </rv>
@@ -4321,26 +4320,26 @@
     <v>637.01</v>
     <v>402.39</v>
     <v>1.0104</v>
-    <v>3.56</v>
-    <v>5.7169999999999999E-3</v>
+    <v>4.93</v>
+    <v>7.9279999999999993E-3</v>
     <v>USD</v>
     <v>Nasdaq Stock Market</v>
     <v>XNAS</v>
-    <v>2E-3</v>
-    <v>627.61</v>
+    <v>1.8E-3</v>
+    <v>627.6</v>
     <v>ETF</v>
-    <v>46048.833621712503</v>
+    <v>46055.684834096872</v>
     <v>43</v>
-    <v>622.12</v>
+    <v>618.70000000000005</v>
     <v>407171619195.83002</v>
     <v>Invesco QQQ Trust 1</v>
-    <v>623.32000000000005</v>
-    <v>622.72</v>
-    <v>626.28</v>
+    <v>618.99</v>
+    <v>621.87</v>
+    <v>626.79999999999995</v>
     <v>QQQ</v>
     <v>Invesco QQQ Trust 1 (XNAS:QQQ)</v>
-    <v>27613933</v>
-    <v>50424109</v>
+    <v>21316141</v>
+    <v>49485835</v>
   </rv>
   <rv s="2">
     <v>44</v>
@@ -4364,26 +4363,26 @@
     <v>496.34</v>
     <v>366.32</v>
     <v>0.8891</v>
-    <v>3.25</v>
-    <v>6.62E-3</v>
+    <v>4.33</v>
+    <v>8.853999999999999E-3</v>
     <v>USD</v>
     <v>NYSE Arca</v>
     <v>ARCX</v>
     <v>1.6000000000000001E-3</v>
-    <v>494.55</v>
+    <v>493.76</v>
     <v>ETF</v>
-    <v>46048.833592592186</v>
+    <v>46055.684822488278</v>
     <v>46</v>
-    <v>491.47</v>
-    <v>44441009524.029999</v>
+    <v>486.99</v>
+    <v>43532474892.239998</v>
     <v>SPDR Dow Jones Indus Avg</v>
-    <v>491.87</v>
-    <v>490.93</v>
-    <v>494.18</v>
+    <v>488.6</v>
+    <v>489.03</v>
+    <v>493.36</v>
     <v>DIA</v>
     <v>SPDR Dow Jones Indus Avg (ARCX:DIA)</v>
-    <v>2743480</v>
-    <v>4709605</v>
+    <v>2945412</v>
+    <v>5515345</v>
   </rv>
   <rv s="2">
     <v>47</v>
@@ -4404,29 +4403,29 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>86.84</v>
+    <v>87.76</v>
     <v>41.1</v>
     <v>1.1644000000000001</v>
-    <v>-0.41</v>
-    <v>-4.7569999999999999E-3</v>
+    <v>-2.2275</v>
+    <v>-2.5666999999999999E-2</v>
     <v>USD</v>
     <v>Nasdaq Stock Market</v>
     <v>XNAS</v>
     <v>7.0999999999999995E-3</v>
-    <v>85.77</v>
+    <v>85.786100000000005</v>
     <v>ETF</v>
-    <v>46048.81162209453</v>
+    <v>46052.885416805468</v>
     <v>49</v>
-    <v>85.77</v>
-    <v>46775464.350000001</v>
+    <v>84.555999999999997</v>
+    <v>50915385.979999997</v>
     <v>FT II:SNet Fut Vhc &amp; Tch</v>
-    <v>85.77</v>
-    <v>86.18</v>
-    <v>85.77</v>
+    <v>85.786100000000005</v>
+    <v>86.783500000000004</v>
+    <v>84.555999999999997</v>
     <v>CARZ</v>
     <v>FT II:SNet Fut Vhc &amp; Tch (XNAS:CARZ)</v>
-    <v>916</v>
-    <v>5524</v>
+    <v>115</v>
+    <v>5508</v>
   </rv>
   <rv s="2">
     <v>50</v>
@@ -6111,7 +6110,7 @@
     <col min="8" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="49" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="33" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -6171,19 +6170,19 @@
       </c>
       <c r="H2" s="20" cm="1">
         <f t="array" aca="1" ref="H2" ca="1">_FV(B2,"Price")</f>
-        <v>186.36009999999999</v>
+        <v>188.99940000000001</v>
       </c>
       <c r="I2" s="20">
         <f ca="1">F2*H2</f>
-        <v>1863601</v>
+        <v>1889994</v>
       </c>
       <c r="J2" s="23">
         <f ca="1">I2-G2</f>
-        <v>1729901</v>
+        <v>1756294</v>
       </c>
       <c r="K2" s="24">
         <f ca="1">J2/G2</f>
-        <v>12.938676140613314</v>
+        <v>13.136080777860883</v>
       </c>
       <c r="M2" t="str" cm="1">
         <f t="array" aca="1" ref="M2" ca="1">_FV(B2,"Ticker symbol",TRUE)</f>
@@ -6215,19 +6214,19 @@
       </c>
       <c r="H3" s="20" cm="1">
         <f t="array" aca="1" ref="H3" ca="1">_FV(B3,"Price")</f>
-        <v>392.9</v>
+        <v>434.75</v>
       </c>
       <c r="I3" s="20">
         <f t="shared" ref="I3:I13" ca="1" si="1">F3*H3</f>
-        <v>275030</v>
+        <v>304325</v>
       </c>
       <c r="J3" s="23">
         <f t="shared" ref="J3:J13" ca="1" si="2">I3-G3</f>
-        <v>216580</v>
+        <v>245875</v>
       </c>
       <c r="K3" s="24">
         <f t="shared" ref="K3:K13" ca="1" si="3">J3/G3</f>
-        <v>3.7053892215568864</v>
+        <v>4.206586826347305</v>
       </c>
       <c r="M3" t="str" cm="1">
         <f t="array" aca="1" ref="M3" ca="1">_FV(B3,"Ticker symbol",TRUE)</f>
@@ -6259,19 +6258,19 @@
       </c>
       <c r="H4" s="20" cm="1">
         <f t="array" aca="1" ref="H4" ca="1">_FV(B4,"Price")</f>
-        <v>223.59</v>
+        <v>237.095</v>
       </c>
       <c r="I4" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>156513</v>
+        <v>165966.5</v>
       </c>
       <c r="J4" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>117103</v>
+        <v>126556.5</v>
       </c>
       <c r="K4" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>2.9714031971580819</v>
+        <v>3.2112788632326819</v>
       </c>
       <c r="M4" t="str" cm="1">
         <f t="array" aca="1" ref="M4" ca="1">_FV(B4,"Ticker symbol",TRUE)</f>
@@ -6303,19 +6302,19 @@
       </c>
       <c r="H5" s="20" cm="1">
         <f t="array" aca="1" ref="H5" ca="1">_FV(B5,"Price")</f>
-        <v>319.375</v>
+        <v>328.43</v>
       </c>
       <c r="I5" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>127750</v>
+        <v>131372</v>
       </c>
       <c r="J5" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>84614</v>
+        <v>88236</v>
       </c>
       <c r="K5" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>1.9615634272997033</v>
+        <v>2.0455304154302669</v>
       </c>
       <c r="M5" t="str" cm="1">
         <f t="array" aca="1" ref="M5" ca="1">_FV(B5,"Ticker symbol",TRUE)</f>
@@ -6347,19 +6346,19 @@
       </c>
       <c r="H6" s="20" cm="1">
         <f t="array" aca="1" ref="H6" ca="1">_FV(B6,"Price")</f>
-        <v>472.53</v>
+        <v>426.19499999999999</v>
       </c>
       <c r="I6" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>189012</v>
+        <v>170478</v>
       </c>
       <c r="J6" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>99276</v>
+        <v>80742</v>
       </c>
       <c r="K6" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>1.1063118480877241</v>
+        <v>0.89977266648836585</v>
       </c>
       <c r="M6" t="str" cm="1">
         <f t="array" aca="1" ref="M6" ca="1">_FV(B6,"Ticker symbol",TRUE)</f>
@@ -6391,19 +6390,19 @@
       </c>
       <c r="H7" s="20" cm="1">
         <f t="array" aca="1" ref="H7" ca="1">_FV(B7,"Price")</f>
-        <v>167.5599</v>
+        <v>150.5</v>
       </c>
       <c r="I7" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>335119.8</v>
+        <v>301000</v>
       </c>
       <c r="J7" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>282439.8</v>
+        <v>248320</v>
       </c>
       <c r="K7" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>5.3614236902050108</v>
+        <v>4.7137433561123769</v>
       </c>
       <c r="M7" t="str" cm="1">
         <f t="array" aca="1" ref="M7" ca="1">_FV(B7,"Ticker symbol",TRUE)</f>
@@ -6435,19 +6434,19 @@
       </c>
       <c r="H8" s="20" cm="1">
         <f t="array" aca="1" ref="H8" ca="1">_FV(B8,"Price")</f>
-        <v>256.2</v>
+        <v>264.37</v>
       </c>
       <c r="I8" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>204960</v>
+        <v>211496</v>
       </c>
       <c r="J8" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>99336</v>
+        <v>105872</v>
       </c>
       <c r="K8" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>0.94046807543740063</v>
+        <v>1.0023479512232067</v>
       </c>
       <c r="M8" t="str" cm="1">
         <f t="array" aca="1" ref="M8" ca="1">_FV(B8,"Ticker symbol",TRUE)</f>
@@ -6479,19 +6478,19 @@
       </c>
       <c r="H9" s="20" cm="1">
         <f t="array" aca="1" ref="H9" ca="1">_FV(B9,"Price")</f>
-        <v>15.065</v>
+        <v>14.85</v>
       </c>
       <c r="I9" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>37662.5</v>
+        <v>37125</v>
       </c>
       <c r="J9" s="23">
         <f ca="1">I9-G9</f>
-        <v>-32587.5</v>
+        <v>-33125</v>
       </c>
       <c r="K9" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>-0.46387900355871886</v>
+        <v>-0.47153024911032027</v>
       </c>
       <c r="M9" t="str" cm="1">
         <f t="array" aca="1" ref="M9" ca="1">_FV(B9,"Ticker symbol",TRUE)</f>
@@ -6523,19 +6522,19 @@
       </c>
       <c r="H10" s="20" cm="1">
         <f t="array" aca="1" ref="H10" ca="1">_FV(B10,"Price")</f>
-        <v>134.91499999999999</v>
+        <v>139.28</v>
       </c>
       <c r="I10" s="20">
         <f ca="1">F10*H10</f>
-        <v>404745</v>
+        <v>417840</v>
       </c>
       <c r="J10" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>256155</v>
+        <v>269250</v>
       </c>
       <c r="K10" s="24">
         <f ca="1">J10/G10</f>
-        <v>1.7239047042196649</v>
+        <v>1.8120331112457098</v>
       </c>
       <c r="M10" t="str" cm="1">
         <f t="array" aca="1" ref="M10" ca="1">_FV(B10,"Ticker symbol",TRUE)</f>
@@ -6567,19 +6566,19 @@
       </c>
       <c r="H11" s="20" cm="1">
         <f t="array" aca="1" ref="H11" ca="1">_FV(B11,"Price")</f>
-        <v>167.06</v>
+        <v>174.4759</v>
       </c>
       <c r="I11" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>200472</v>
+        <v>209371.08</v>
       </c>
       <c r="J11" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>86016</v>
+        <v>94915.079999999987</v>
       </c>
       <c r="K11" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>0.75152023485007335</v>
+        <v>0.82927133570979228</v>
       </c>
       <c r="M11" t="str" cm="1">
         <f t="array" aca="1" ref="M11" ca="1">_FV(B11,"Ticker symbol",TRUE)</f>
@@ -6611,19 +6610,19 @@
       </c>
       <c r="H12" s="20" cm="1">
         <f t="array" aca="1" ref="H12" ca="1">_FV(B12,"Price")</f>
-        <v>56.72</v>
+        <v>56.55</v>
       </c>
       <c r="I12" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>226880</v>
+        <v>226200</v>
       </c>
       <c r="J12" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>135320</v>
+        <v>134640</v>
       </c>
       <c r="K12" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>1.4779379641764963</v>
+        <v>1.4705111402359108</v>
       </c>
       <c r="M12" t="str" cm="1">
         <f t="array" aca="1" ref="M12" ca="1">_FV(B12,"Ticker symbol",TRUE)</f>
@@ -6655,19 +6654,19 @@
       </c>
       <c r="H13" s="20" cm="1">
         <f t="array" aca="1" ref="H13" ca="1">_FV(B13,"Price")</f>
-        <v>52.06</v>
+        <v>53.765000000000001</v>
       </c>
       <c r="I13" s="20">
         <f t="shared" ca="1" si="1"/>
-        <v>260300</v>
+        <v>268825</v>
       </c>
       <c r="J13" s="23">
         <f t="shared" ca="1" si="2"/>
-        <v>209450</v>
+        <v>217975</v>
       </c>
       <c r="K13" s="24">
         <f t="shared" ca="1" si="3"/>
-        <v>4.1189773844641104</v>
+        <v>4.2866273352999018</v>
       </c>
       <c r="M13" t="str" cm="1">
         <f t="array" aca="1" ref="M13" ca="1">_FV(B13,"Ticker symbol",TRUE)</f>
@@ -6695,6 +6694,10 @@
         <v>0.15</v>
       </c>
       <c r="G16" s="19"/>
+      <c r="I16">
+        <f>+J17</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
@@ -6748,31 +6751,31 @@
       </c>
       <c r="D20" s="25">
         <f ca="1">SUM(I2:I13)</f>
-        <v>4282045.3</v>
+        <v>4333992.58</v>
       </c>
       <c r="E20" s="25">
         <f ca="1">D20+C20</f>
-        <v>4283603.3</v>
+        <v>4335550.58</v>
       </c>
       <c r="F20" s="25">
         <f ca="1">SUM(J2:J13)</f>
-        <v>3283603.3</v>
+        <v>3335550.58</v>
       </c>
       <c r="G20" s="26">
-        <f ca="1">(F20-A20)/A20</f>
-        <v>2.2836032999999998</v>
+        <f ca="1">(E20-A20)/A20</f>
+        <v>3.33555058</v>
       </c>
       <c r="H20" s="25">
         <f ca="1">B16*F20</f>
-        <v>492540.49499999994</v>
+        <v>500332.587</v>
       </c>
       <c r="I20" s="25">
         <f ca="1">E20-H20</f>
-        <v>3791062.8049999997</v>
+        <v>3835217.9930000002</v>
       </c>
       <c r="J20" s="26">
-        <f ca="1">(F20-H20-A20)/A20</f>
-        <v>1.7910628049999997</v>
+        <f ca="1">(I20-A20)/A20</f>
+        <v>2.8352179930000001</v>
       </c>
     </row>
   </sheetData>
@@ -7050,7 +7053,7 @@
     <col min="15" max="15" width="15.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="81" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="65" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>14</v>
       </c>
@@ -7117,35 +7120,35 @@
       </c>
       <c r="G2" s="20" cm="1">
         <f t="array" aca="1" ref="G2" ca="1">_FV(B2,"Price")</f>
-        <v>638.83000000000004</v>
+        <v>641.03</v>
       </c>
       <c r="H2" s="20">
         <f ca="1">G2*D2</f>
-        <v>1795751.1300000001</v>
+        <v>1801935.3299999998</v>
       </c>
       <c r="I2" s="20">
         <f ca="1">H2+F2</f>
-        <v>1795962.7600000002</v>
+        <v>1802146.96</v>
       </c>
       <c r="J2" s="23">
         <f ca="1">H2-E2</f>
-        <v>795962.76000000013</v>
+        <v>802146.95999999985</v>
       </c>
       <c r="K2" s="24">
-        <f ca="1">J2/E2</f>
-        <v>0.79613124525543355</v>
+        <f ca="1">(I2-1000000)/1000000</f>
+        <v>0.80214695999999996</v>
       </c>
       <c r="L2" s="23">
         <f ca="1">J2*0.15</f>
-        <v>119394.41400000002</v>
+        <v>120322.04399999997</v>
       </c>
       <c r="M2" s="23">
         <f ca="1">I2-L2</f>
-        <v>1676568.3460000001</v>
+        <v>1681824.916</v>
       </c>
       <c r="N2" s="24">
-        <f ca="1">(J2-L2)/E2</f>
-        <v>0.6767115584671185</v>
+        <f ca="1">(M2-1000000)/1000000</f>
+        <v>0.68182491599999995</v>
       </c>
       <c r="O2" s="21"/>
     </row>
@@ -7172,35 +7175,35 @@
       </c>
       <c r="G3" s="20" cm="1">
         <f t="array" aca="1" ref="G3" ca="1">_FV(B3,"Price")</f>
-        <v>626.28</v>
+        <v>626.79999999999995</v>
       </c>
       <c r="H3" s="20">
         <f t="shared" ref="H3:H5" ca="1" si="2">G3*D3</f>
-        <v>1933952.64</v>
+        <v>1935558.4</v>
       </c>
       <c r="I3" s="20">
         <f t="shared" ref="I3:I5" ca="1" si="3">H3+F3</f>
-        <v>1934150.88</v>
+        <v>1935756.6400000001</v>
       </c>
       <c r="J3" s="23">
-        <f t="shared" ref="J3:J5" ca="1" si="4">H3-E3</f>
-        <v>934150.88</v>
+        <f ca="1">H3-E3</f>
+        <v>935756.64</v>
       </c>
       <c r="K3" s="24">
-        <f ca="1">J3/E3</f>
-        <v>0.93433610278901702</v>
+        <f t="shared" ref="K3:K5" ca="1" si="4">(I3-1000000)/1000000</f>
+        <v>0.93575664000000014</v>
       </c>
       <c r="L3" s="23">
-        <f t="shared" ref="L3:L5" ca="1" si="5">J3*0.15</f>
-        <v>140122.63199999998</v>
+        <f ca="1">J3*0.15</f>
+        <v>140363.49599999998</v>
       </c>
       <c r="M3" s="23">
-        <f t="shared" ref="M3:M5" ca="1" si="6">I3-L3</f>
-        <v>1794028.2479999999</v>
+        <f t="shared" ref="M3:M5" ca="1" si="5">I3-L3</f>
+        <v>1795393.1440000001</v>
       </c>
       <c r="N3" s="24">
-        <f t="shared" ref="N3:N5" ca="1" si="7">(J3-L3)/E3</f>
-        <v>0.79418568737066442</v>
+        <f t="shared" ref="N3:N5" ca="1" si="6">(M3-1000000)/1000000</f>
+        <v>0.79539314400000005</v>
       </c>
       <c r="O3" s="21"/>
     </row>
@@ -7227,35 +7230,35 @@
       </c>
       <c r="G4" s="20" cm="1">
         <f t="array" aca="1" ref="G4" ca="1">_FV(B4,"Price")</f>
-        <v>494.18</v>
+        <v>493.36</v>
       </c>
       <c r="H4" s="20">
         <f t="shared" ca="1" si="2"/>
-        <v>1584835.26</v>
+        <v>1582205.52</v>
       </c>
       <c r="I4" s="20">
         <f ca="1">H4+F4</f>
-        <v>1584988.87</v>
+        <v>1582359.1300000001</v>
       </c>
       <c r="J4" s="23">
+        <f t="shared" ref="J4:J5" ca="1" si="7">H4-E4</f>
+        <v>582359.13000000012</v>
+      </c>
+      <c r="K4" s="24">
         <f t="shared" ca="1" si="4"/>
-        <v>584988.87000000011</v>
-      </c>
-      <c r="K4" s="24">
-        <f t="shared" ref="K3:K5" ca="1" si="8">J4/E4</f>
-        <v>0.58507874394585768</v>
+        <v>0.58235913000000017</v>
       </c>
       <c r="L4" s="23">
+        <f ca="1">J4*0.15</f>
+        <v>87353.869500000015</v>
+      </c>
+      <c r="M4" s="23">
         <f t="shared" ca="1" si="5"/>
-        <v>87748.330500000011</v>
-      </c>
-      <c r="M4" s="23">
+        <v>1495005.2605000001</v>
+      </c>
+      <c r="N4" s="24">
         <f t="shared" ca="1" si="6"/>
-        <v>1497240.5395000002</v>
-      </c>
-      <c r="N4" s="24">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.497316932353979</v>
+        <v>0.4950052605000001</v>
       </c>
       <c r="O4" s="21"/>
     </row>
@@ -7282,35 +7285,35 @@
       </c>
       <c r="G5" s="20" cm="1">
         <f t="array" aca="1" ref="G5" ca="1">_FV(B5,"Price")</f>
-        <v>85.77</v>
+        <v>84.555999999999997</v>
       </c>
       <c r="H5" s="20">
         <f t="shared" ca="1" si="2"/>
-        <v>1486222.5599999998</v>
+        <v>1465186.368</v>
       </c>
       <c r="I5" s="20">
         <f t="shared" ca="1" si="3"/>
-        <v>1486223.6799999997</v>
+        <v>1465187.4879999999</v>
       </c>
       <c r="J5" s="23">
+        <f t="shared" ca="1" si="7"/>
+        <v>465187.48800000001</v>
+      </c>
+      <c r="K5" s="24">
         <f t="shared" ca="1" si="4"/>
-        <v>486223.67999999982</v>
-      </c>
-      <c r="K5" s="24">
-        <f t="shared" ca="1" si="8"/>
-        <v>0.48622422457113135</v>
+        <v>0.46518748799999987</v>
       </c>
       <c r="L5" s="23">
+        <f t="shared" ref="L5" ca="1" si="8">J5*0.15</f>
+        <v>69778.123200000002</v>
+      </c>
+      <c r="M5" s="23">
         <f t="shared" ca="1" si="5"/>
-        <v>72933.551999999967</v>
-      </c>
-      <c r="M5" s="23">
+        <v>1395409.3647999999</v>
+      </c>
+      <c r="N5" s="24">
         <f t="shared" ca="1" si="6"/>
-        <v>1413290.1279999998</v>
-      </c>
-      <c r="N5" s="24">
-        <f t="shared" ca="1" si="7"/>
-        <v>0.41329059088546166</v>
+        <v>0.39540936479999989</v>
       </c>
       <c r="O5" s="21"/>
     </row>
@@ -7324,28 +7327,22 @@
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
       <c r="G6" s="8"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="36">
+      <c r="H6" s="33"/>
+      <c r="I6" s="35">
         <f ca="1">'Main Analysis'!E20</f>
-        <v>4283603.3</v>
+        <v>4335550.58</v>
       </c>
       <c r="J6" s="3"/>
-      <c r="K6" s="35">
+      <c r="K6" s="34">
         <f ca="1">'Main Analysis'!G20</f>
-        <v>2.2836032999999998</v>
+        <v>3.33555058</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
-      <c r="N6" s="35"/>
+      <c r="N6" s="34"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="33"/>
+      <c r="H7" s="32"/>
       <c r="N7" s="19"/>
     </row>
     <row r="12" spans="1:15" ht="29" x14ac:dyDescent="0.35">

</xml_diff>